<commit_message>
fitted end of day
</commit_message>
<xml_diff>
--- a/BeatnotePostHotCell/AllFitsF1=3_playing with.xlsx
+++ b/BeatnotePostHotCell/AllFitsF1=3_playing with.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\nas01.itap.purdue.edu\puhome\desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\BeatnotePostHotCell\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF320C90-E5DA-41F4-93D7-1188D7FEA2C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A4447D4-8053-4676-AC00-7E68C4D6F1B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10678,11 +10678,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'894'!$C$3</c:f>
+              <c:f>'894'!$G$3</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Jun09,2026</c:v>
+                  <c:v>Jun15,2030</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -10830,69 +10830,102 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'894'!$C$4:$C$233</c:f>
+              <c:f>'894'!$G$4:$G$233</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="230"/>
                 <c:pt idx="0">
-                  <c:v>8.53551089338964</c:v>
+                  <c:v>15.5831740366148</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.2121360213246692</c:v>
+                  <c:v>15.6181213588261</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.3727208112640206</c:v>
+                  <c:v>15.471660411280601</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.4364141305933895</c:v>
+                  <c:v>15.4286358328345</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.4084015562695207</c:v>
+                  <c:v>15.725390191826</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.5099572412062301</c:v>
+                  <c:v>15.6295450777592</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>8.4321434520724008</c:v>
+                  <c:v>15.5447105698267</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>8.4721216638779193</c:v>
+                  <c:v>15.641779033917301</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8.4953666075608503</c:v>
+                  <c:v>15.560241393406899</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.7711252103094601</c:v>
+                  <c:v>15.6798903930978</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>8.5801266895029205</c:v>
+                  <c:v>15.5257705053734</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>8.5783681642005494</c:v>
+                  <c:v>15.5068553708303</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>8.6129268121772302</c:v>
+                  <c:v>15.7245514226287</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>8.6349505815443095</c:v>
+                  <c:v>15.653971830187899</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>8.5827352500219707</c:v>
+                  <c:v>15.585241971938</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>8.6784045244654298</c:v>
+                  <c:v>15.591441713773801</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>8.5889121451567796</c:v>
+                  <c:v>15.513624662526899</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>8.2237273067390202</c:v>
+                  <c:v>15.550450799138201</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>8.26640584418465</c:v>
+                  <c:v>15.5999990421973</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>8.2614937671479094</c:v>
+                  <c:v>15.5612294230614</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>15.389959627991299</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>15.6769168147221</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>15.516217850365001</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>15.4712021433598</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>15.4267437621642</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>15.363023447442201</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>15.4784018893041</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>15.598700910453401</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>15.699463941581101</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>15.751226314712399</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>15.601321813860199</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -14987,16 +15020,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>171449</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>233632</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>107830</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:colOff>560359</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>512191</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -15025,14 +15058,14 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>161925</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>352425</xdr:rowOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>476250</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -15213,16 +15246,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>514350</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>71437</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>147637</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>485775</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>109537</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -19196,7 +19229,7 @@
         <v>0.82580237252011701</v>
       </c>
       <c r="C2">
-        <f t="shared" ref="C2:K2" si="1">100*C1/AVERAGE(C4:C39)</f>
+        <f t="shared" ref="C2:J2" si="1">100*C1/AVERAGE(C4:C39)</f>
         <v>0.41179120150630028</v>
       </c>
       <c r="D2">

</xml_diff>

<commit_message>
Need to redo fittings
</commit_message>
<xml_diff>
--- a/BeatnotePostHotCell/AllFitsF1=3_playing with.xlsx
+++ b/BeatnotePostHotCell/AllFitsF1=3_playing with.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\BeatnotePostHotCell\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wolfwalker\Documents\git\6s7p\BeatnotePostHotCell\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A4447D4-8053-4676-AC00-7E68C4D6F1B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5562D9B-800E-4A8B-A55A-17EAFFE389C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Together" sheetId="1" r:id="rId1"/>
@@ -30,9 +30,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -2662,6 +2659,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2669,7 +2667,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4661,6 +4658,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4668,7 +4666,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4953,6 +4950,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4960,7 +4958,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7533,6 +7530,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7540,7 +7538,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8001,6 +7998,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8008,7 +8006,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10581,6 +10578,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10588,7 +10586,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11082,6 +11079,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11089,7 +11087,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -15020,16 +15017,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>233632</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>107830</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>491226</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>527170</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>560359</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>512191</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>117056</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>380399</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -15546,13 +15543,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P233"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P295"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -15593,7 +15590,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -15647,7 +15644,7 @@
         <v>5.1155359965755959E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -15701,7 +15698,7 @@
         <v>1.2279085192200808E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -15715,7 +15712,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -15726,7 +15723,7 @@
         <v>0.17477778117201601</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -15737,7 +15734,7 @@
         <v>0.17496986858800301</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -15748,7 +15745,7 @@
         <v>0.39075425090921301</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -15759,7 +15756,7 @@
         <v>0.39090251610402299</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -15770,7 +15767,7 @@
         <v>0.38163793874347302</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -15781,7 +15778,7 @@
         <v>0.38646897393750201</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -15792,7 +15789,7 @@
         <v>0.38820632020412599</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -15803,7 +15800,7 @@
         <v>0.391100077546855</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
@@ -15814,7 +15811,7 @@
         <v>0.37812534333091802</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -15825,7 +15822,7 @@
         <v>0.38449528426413199</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -15836,7 +15833,7 @@
         <v>0.38779470041263903</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
@@ -15847,7 +15844,7 @@
         <v>0.378248054436716</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
@@ -15858,7 +15855,7 @@
         <v>0.388322173460803</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
@@ -15869,7 +15866,7 @@
         <v>0.38881861759339797</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
@@ -15880,7 +15877,7 @@
         <v>0.39254780032303299</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
@@ -15891,7 +15888,7 @@
         <v>0.38860291038577099</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
@@ -15902,7 +15899,7 @@
         <v>0.391344107724999</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -15913,7 +15910,7 @@
         <v>0.39401793952400199</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>22</v>
       </c>
@@ -15924,7 +15921,7 @@
         <v>0.398157579716993</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>23</v>
       </c>
@@ -15935,7 +15932,7 @@
         <v>0.38710256673105198</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>24</v>
       </c>
@@ -15946,7 +15943,7 @@
         <v>0.18265936593662399</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>25</v>
       </c>
@@ -15957,7 +15954,7 @@
         <v>0.17720413354468001</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
@@ -15968,7 +15965,7 @@
         <v>0.183642067498062</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
@@ -15979,7 +15976,7 @@
         <v>0.18126642652018499</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>28</v>
       </c>
@@ -15990,7 +15987,7 @@
         <v>0.17863631678412401</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>29</v>
       </c>
@@ -16001,7 +15998,7 @@
         <v>0.18200369359492499</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>30</v>
       </c>
@@ -16012,7 +16009,7 @@
         <v>0.18140063454570701</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>31</v>
       </c>
@@ -16023,7 +16020,7 @@
         <v>0.14198189433295499</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>32</v>
       </c>
@@ -16034,7 +16031,7 @@
         <v>0.14200693706074399</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>33</v>
       </c>
@@ -16045,7 +16042,7 @@
         <v>0.13879302222888601</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>34</v>
       </c>
@@ -16056,7 +16053,7 @@
         <v>0.14134057599559999</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>35</v>
       </c>
@@ -16067,7 +16064,7 @@
         <v>0.14287369952523299</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>36</v>
       </c>
@@ -16078,7 +16075,7 @@
         <v>0.14242039757473199</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>37</v>
       </c>
@@ -16089,7 +16086,7 @@
         <v>0.13513280226965799</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>38</v>
       </c>
@@ -16100,7 +16097,7 @@
         <v>0.13504563445130599</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>39</v>
       </c>
@@ -16111,7 +16108,7 @@
         <v>0.13859780418944301</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>40</v>
       </c>
@@ -16122,7 +16119,7 @@
         <v>0.13768382280778599</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>41</v>
       </c>
@@ -16133,7 +16130,7 @@
         <v>0.137341027012235</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>42</v>
       </c>
@@ -16144,7 +16141,7 @@
         <v>0.14146322755453</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>43</v>
       </c>
@@ -16155,7 +16152,7 @@
         <v>0.1440878295095</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>44</v>
       </c>
@@ -16166,7 +16163,7 @@
         <v>0.139203017324112</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>45</v>
       </c>
@@ -16177,7 +16174,7 @@
         <v>0.14444988833485001</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>46</v>
       </c>
@@ -16188,7 +16185,7 @@
         <v>0.14486186097849299</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>47</v>
       </c>
@@ -16199,7 +16196,7 @@
         <v>0.14493175120103199</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>48</v>
       </c>
@@ -16210,7 +16207,7 @@
         <v>0.14335784354365599</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>49</v>
       </c>
@@ -16221,7 +16218,7 @@
         <v>0.14372426788936199</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>50</v>
       </c>
@@ -16232,7 +16229,7 @@
         <v>0.140914458888726</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>51</v>
       </c>
@@ -16243,7 +16240,7 @@
         <v>0.144559929539015</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>52</v>
       </c>
@@ -16254,7 +16251,7 @@
         <v>0.13911305366694399</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>53</v>
       </c>
@@ -16265,7 +16262,7 @@
         <v>0.136881983671574</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>54</v>
       </c>
@@ -16276,7 +16273,7 @@
         <v>0.135891683439223</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>55</v>
       </c>
@@ -16287,7 +16284,7 @@
         <v>0.134600217130598</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>58</v>
       </c>
@@ -16298,7 +16295,7 @@
         <v>0.117218052017694</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>59</v>
       </c>
@@ -16309,7 +16306,7 @@
         <v>0.116738218899043</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>60</v>
       </c>
@@ -16320,7 +16317,7 @@
         <v>0.116641895814922</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>61</v>
       </c>
@@ -16331,7 +16328,7 @@
         <v>0.117986722306339</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>62</v>
       </c>
@@ -16342,7 +16339,7 @@
         <v>0.116363944216263</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>63</v>
       </c>
@@ -16353,7 +16350,7 @@
         <v>0.117960737624138</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>64</v>
       </c>
@@ -16364,7 +16361,7 @@
         <v>0.11777189549636199</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>65</v>
       </c>
@@ -16375,7 +16372,7 @@
         <v>0.118362346500101</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>66</v>
       </c>
@@ -16386,7 +16383,7 @@
         <v>0.11875028071223</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>67</v>
       </c>
@@ -16397,7 +16394,7 @@
         <v>0.118209453954305</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>68</v>
       </c>
@@ -16408,7 +16405,7 @@
         <v>0.116577694816434</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>69</v>
       </c>
@@ -16419,7 +16416,7 @@
         <v>0.117670638852321</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>70</v>
       </c>
@@ -16430,7 +16427,7 @@
         <v>0.118098845799444</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>71</v>
       </c>
@@ -16441,7 +16438,7 @@
         <v>0.11655919684067299</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>72</v>
       </c>
@@ -16452,7 +16449,7 @@
         <v>0.118487075826876</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>73</v>
       </c>
@@ -16463,7 +16460,7 @@
         <v>0.117049111989703</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>74</v>
       </c>
@@ -16474,7 +16471,7 @@
         <v>0.116964493443121</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>75</v>
       </c>
@@ -16485,7 +16482,7 @@
         <v>0.1174932059815</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>76</v>
       </c>
@@ -16496,7 +16493,7 @@
         <v>0.118724780988732</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>77</v>
       </c>
@@ -16507,7 +16504,7 @@
         <v>0.11857414162119</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>78</v>
       </c>
@@ -16518,7 +16515,7 @@
         <v>0.116857985488521</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>79</v>
       </c>
@@ -16529,7 +16526,7 @@
         <v>0.117839930521939</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>80</v>
       </c>
@@ -16540,7 +16537,7 @@
         <v>0.116123290748398</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>81</v>
       </c>
@@ -16551,7 +16548,7 @@
         <v>0.116339626646247</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>82</v>
       </c>
@@ -16562,7 +16559,7 @@
         <v>0.118521454357363</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>83</v>
       </c>
@@ -16573,7 +16570,7 @@
         <v>0.117743388207075</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>84</v>
       </c>
@@ -16584,7 +16581,7 @@
         <v>0.116823099810358</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>85</v>
       </c>
@@ -16595,7 +16592,7 @@
         <v>0.118509294607666</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>86</v>
       </c>
@@ -16606,7 +16603,7 @@
         <v>0.118631007440724</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>87</v>
       </c>
@@ -16617,7 +16614,7 @@
         <v>0.117484320873481</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>88</v>
       </c>
@@ -16628,7 +16625,7 @@
         <v>0.118251546607688</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>89</v>
       </c>
@@ -16639,7 +16636,7 @@
         <v>0.118181098472526</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>90</v>
       </c>
@@ -16650,7 +16647,7 @@
         <v>8.9287039240001795E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>91</v>
       </c>
@@ -16661,7 +16658,7 @@
         <v>8.9953273584561996E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>92</v>
       </c>
@@ -16672,7 +16669,7 @@
         <v>9.1230909809772498E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>93</v>
       </c>
@@ -16683,7 +16680,7 @@
         <v>9.0037965159722497E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>94</v>
       </c>
@@ -16694,7 +16691,7 @@
         <v>9.2063662732121604E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>95</v>
       </c>
@@ -16705,7 +16702,7 @@
         <v>9.0566169869859395E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>96</v>
       </c>
@@ -16716,7 +16713,7 @@
         <v>9.1281359996997199E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>97</v>
       </c>
@@ -16727,7 +16724,7 @@
         <v>9.0246189977935598E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>98</v>
       </c>
@@ -16738,7 +16735,7 @@
         <v>8.7987770056780296E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>99</v>
       </c>
@@ -16749,7 +16746,7 @@
         <v>9.1038024594974204E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>100</v>
       </c>
@@ -16760,7 +16757,7 @@
         <v>9.0356969610468907E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>101</v>
       </c>
@@ -16771,7 +16768,7 @@
         <v>8.9055177802521202E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>102</v>
       </c>
@@ -16782,7 +16779,7 @@
         <v>9.0556231765949805E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>103</v>
       </c>
@@ -16793,7 +16790,7 @@
         <v>9.1259865204828206E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>104</v>
       </c>
@@ -16804,7 +16801,7 @@
         <v>8.8371089308141498E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>105</v>
       </c>
@@ -16815,7 +16812,7 @@
         <v>8.9886315679026302E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>106</v>
       </c>
@@ -16826,7 +16823,7 @@
         <v>0.22378459935658199</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>107</v>
       </c>
@@ -16837,7 +16834,7 @@
         <v>0.228434718604688</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>108</v>
       </c>
@@ -16848,7 +16845,7 @@
         <v>0.221372998488612</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>109</v>
       </c>
@@ -16859,7 +16856,7 @@
         <v>0.225975457594905</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>110</v>
       </c>
@@ -16870,7 +16867,7 @@
         <v>0.225216837741747</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>111</v>
       </c>
@@ -16881,7 +16878,7 @@
         <v>0.229746279532067</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>112</v>
       </c>
@@ -16892,7 +16889,7 @@
         <v>0.22722518963626401</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>113</v>
       </c>
@@ -16903,7 +16900,7 @@
         <v>0.222965184868961</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>114</v>
       </c>
@@ -16914,7 +16911,7 @@
         <v>0.22898718060617901</v>
       </c>
     </row>
-    <row r="114" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>115</v>
       </c>
@@ -16925,7 +16922,7 @@
         <v>0.22580668748875701</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>116</v>
       </c>
@@ -16936,7 +16933,7 @@
         <v>0.231594890582631</v>
       </c>
     </row>
-    <row r="116" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>117</v>
       </c>
@@ -16947,7 +16944,7 @@
         <v>0.224583618990919</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>118</v>
       </c>
@@ -16958,7 +16955,7 @@
         <v>0.23249128317182099</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>119</v>
       </c>
@@ -16969,7 +16966,7 @@
         <v>0.23073510515949899</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>120</v>
       </c>
@@ -16980,7 +16977,7 @@
         <v>0.229179326874075</v>
       </c>
     </row>
-    <row r="120" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>121</v>
       </c>
@@ -16991,7 +16988,7 @@
         <v>0.226024665246639</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>122</v>
       </c>
@@ -17002,7 +16999,7 @@
         <v>0.22988414195496401</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>123</v>
       </c>
@@ -17013,7 +17010,7 @@
         <v>0.22795719930278499</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>124</v>
       </c>
@@ -17024,7 +17021,7 @@
         <v>0.227267035209756</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>125</v>
       </c>
@@ -17035,7 +17032,7 @@
         <v>0.22728875634974799</v>
       </c>
     </row>
-    <row r="125" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>126</v>
       </c>
@@ -17046,7 +17043,7 @@
         <v>0.22819660608103401</v>
       </c>
     </row>
-    <row r="126" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>127</v>
       </c>
@@ -17057,7 +17054,7 @@
         <v>0.22449918198189101</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>128</v>
       </c>
@@ -17068,7 +17065,7 @@
         <v>0.22352994908158599</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>129</v>
       </c>
@@ -17079,7 +17076,7 @@
         <v>0.22753327784977401</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>130</v>
       </c>
@@ -17090,7 +17087,7 @@
         <v>0.22784419865740199</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>131</v>
       </c>
@@ -17101,7 +17098,7 @@
         <v>0.225433003733543</v>
       </c>
     </row>
-    <row r="131" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>132</v>
       </c>
@@ -17112,7 +17109,7 @@
         <v>0.22712348211729699</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>133</v>
       </c>
@@ -17123,7 +17120,7 @@
         <v>0.22894109101944199</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>134</v>
       </c>
@@ -17134,7 +17131,7 @@
         <v>0.23027592968354901</v>
       </c>
     </row>
-    <row r="134" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>135</v>
       </c>
@@ -17145,7 +17142,7 @@
         <v>0.22733899516780401</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>136</v>
       </c>
@@ -17156,7 +17153,7 @@
         <v>0.22718964047891599</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>137</v>
       </c>
@@ -17167,7 +17164,7 @@
         <v>0.22249606599096799</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>138</v>
       </c>
@@ -17178,7 +17175,7 @@
         <v>0.22770140189949001</v>
       </c>
     </row>
-    <row r="138" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>139</v>
       </c>
@@ -17189,7 +17186,7 @@
         <v>0.22467693879523801</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>140</v>
       </c>
@@ -17200,7 +17197,7 @@
         <v>0.22590951148508701</v>
       </c>
     </row>
-    <row r="140" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>141</v>
       </c>
@@ -17211,7 +17208,7 @@
         <v>0.22795873224990801</v>
       </c>
     </row>
-    <row r="141" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>142</v>
       </c>
@@ -17222,7 +17219,7 @@
         <v>0.26064960163891099</v>
       </c>
     </row>
-    <row r="142" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>143</v>
       </c>
@@ -17233,7 +17230,7 @@
         <v>0.25338188968269398</v>
       </c>
     </row>
-    <row r="143" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>144</v>
       </c>
@@ -17244,7 +17241,7 @@
         <v>0.25038094455952498</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>145</v>
       </c>
@@ -17255,7 +17252,7 @@
         <v>0.256215228918099</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>146</v>
       </c>
@@ -17266,7 +17263,7 @@
         <v>0.25483329669185101</v>
       </c>
     </row>
-    <row r="146" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>147</v>
       </c>
@@ -17277,7 +17274,7 @@
         <v>0.25854387484878599</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>148</v>
       </c>
@@ -17288,7 +17285,7 @@
         <v>0.25519336396030601</v>
       </c>
     </row>
-    <row r="148" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>149</v>
       </c>
@@ -17299,7 +17296,7 @@
         <v>0.25663303680948102</v>
       </c>
     </row>
-    <row r="149" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>150</v>
       </c>
@@ -17310,7 +17307,7 @@
         <v>0.25601459599486398</v>
       </c>
     </row>
-    <row r="150" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>151</v>
       </c>
@@ -17321,7 +17318,7 @@
         <v>0.25648553124648299</v>
       </c>
     </row>
-    <row r="151" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>152</v>
       </c>
@@ -17332,7 +17329,7 @@
         <v>0.25339182435774998</v>
       </c>
     </row>
-    <row r="152" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>153</v>
       </c>
@@ -17343,7 +17340,7 @@
         <v>0.26261256236820102</v>
       </c>
     </row>
-    <row r="153" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>154</v>
       </c>
@@ -17354,7 +17351,7 @@
         <v>0.25914013258546797</v>
       </c>
     </row>
-    <row r="154" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>155</v>
       </c>
@@ -17365,7 +17362,7 @@
         <v>0.25187380012057398</v>
       </c>
     </row>
-    <row r="155" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>156</v>
       </c>
@@ -17376,7 +17373,7 @@
         <v>0.25861462842520899</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>157</v>
       </c>
@@ -17387,7 +17384,7 @@
         <v>0.26412000142144099</v>
       </c>
     </row>
-    <row r="157" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>158</v>
       </c>
@@ -17398,7 +17395,7 @@
         <v>0.25505739125523702</v>
       </c>
     </row>
-    <row r="158" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>159</v>
       </c>
@@ -17409,7 +17406,7 @@
         <v>0.25268334549192301</v>
       </c>
     </row>
-    <row r="159" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>160</v>
       </c>
@@ -17420,7 +17417,7 @@
         <v>0.254203134019032</v>
       </c>
     </row>
-    <row r="160" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>161</v>
       </c>
@@ -17431,7 +17428,7 @@
         <v>0.25355249186689299</v>
       </c>
     </row>
-    <row r="161" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>162</v>
       </c>
@@ -17442,7 +17439,7 @@
         <v>0.258640908855092</v>
       </c>
     </row>
-    <row r="162" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>163</v>
       </c>
@@ -17453,7 +17450,7 @@
         <v>0.25176887581155899</v>
       </c>
     </row>
-    <row r="163" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>164</v>
       </c>
@@ -17464,7 +17461,7 @@
         <v>0.25436276153236997</v>
       </c>
     </row>
-    <row r="164" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>165</v>
       </c>
@@ -17475,7 +17472,7 @@
         <v>0.25848980394328103</v>
       </c>
     </row>
-    <row r="165" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>166</v>
       </c>
@@ -17486,7 +17483,7 @@
         <v>0.25493042534243598</v>
       </c>
     </row>
-    <row r="166" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>167</v>
       </c>
@@ -17497,7 +17494,7 @@
         <v>0.25702073078272197</v>
       </c>
     </row>
-    <row r="167" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>168</v>
       </c>
@@ -17508,7 +17505,7 @@
         <v>0.25281370286486299</v>
       </c>
     </row>
-    <row r="168" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>169</v>
       </c>
@@ -17519,7 +17516,7 @@
         <v>0.25787828139437702</v>
       </c>
     </row>
-    <row r="169" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>170</v>
       </c>
@@ -17530,7 +17527,7 @@
         <v>0.255030114263046</v>
       </c>
     </row>
-    <row r="170" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>171</v>
       </c>
@@ -17541,7 +17538,7 @@
         <v>0.25326708245889501</v>
       </c>
     </row>
-    <row r="171" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>172</v>
       </c>
@@ -17552,7 +17549,7 @@
         <v>0.25901851572451601</v>
       </c>
     </row>
-    <row r="172" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>173</v>
       </c>
@@ -17563,7 +17560,7 @@
         <v>0.25402214979933802</v>
       </c>
     </row>
-    <row r="173" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>174</v>
       </c>
@@ -17574,7 +17571,7 @@
         <v>0.25207440807669201</v>
       </c>
     </row>
-    <row r="174" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>175</v>
       </c>
@@ -17585,7 +17582,7 @@
         <v>0.25648835225167999</v>
       </c>
     </row>
-    <row r="175" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>176</v>
       </c>
@@ -17596,7 +17593,7 @@
         <v>0.25619702232418301</v>
       </c>
     </row>
-    <row r="176" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>177</v>
       </c>
@@ -17607,7 +17604,7 @@
         <v>0.256904989972564</v>
       </c>
     </row>
-    <row r="177" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>178</v>
       </c>
@@ -17618,7 +17615,7 @@
         <v>0.25656545981822299</v>
       </c>
     </row>
-    <row r="178" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>179</v>
       </c>
@@ -17629,7 +17626,7 @@
         <v>0.25471437628790899</v>
       </c>
     </row>
-    <row r="179" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>180</v>
       </c>
@@ -17640,7 +17637,7 @@
         <v>0.25564492601438199</v>
       </c>
     </row>
-    <row r="180" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>181</v>
       </c>
@@ -17651,7 +17648,7 @@
         <v>0.26266359379455601</v>
       </c>
     </row>
-    <row r="181" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>182</v>
       </c>
@@ -17662,7 +17659,7 @@
         <v>0.25914186884267898</v>
       </c>
     </row>
-    <row r="182" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>183</v>
       </c>
@@ -17673,7 +17670,7 @@
         <v>0.25621155685651098</v>
       </c>
     </row>
-    <row r="183" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>184</v>
       </c>
@@ -17684,7 +17681,7 @@
         <v>0.25866494788723898</v>
       </c>
     </row>
-    <row r="184" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>185</v>
       </c>
@@ -17695,7 +17692,7 @@
         <v>0.25801756322347102</v>
       </c>
     </row>
-    <row r="185" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>186</v>
       </c>
@@ -17706,7 +17703,7 @@
         <v>0.25944545650678502</v>
       </c>
     </row>
-    <row r="186" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>187</v>
       </c>
@@ -17717,7 +17714,7 @@
         <v>0.25336488450504602</v>
       </c>
     </row>
-    <row r="187" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>188</v>
       </c>
@@ -17728,7 +17725,7 @@
         <v>0.261553420142073</v>
       </c>
     </row>
-    <row r="188" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>189</v>
       </c>
@@ -17739,7 +17736,7 @@
         <v>0.26019522603942802</v>
       </c>
     </row>
-    <row r="189" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>190</v>
       </c>
@@ -17750,7 +17747,7 @@
         <v>0.25868729407005198</v>
       </c>
     </row>
-    <row r="190" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>191</v>
       </c>
@@ -17761,7 +17758,7 @@
         <v>0.25516460879894798</v>
       </c>
     </row>
-    <row r="191" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>192</v>
       </c>
@@ -17772,7 +17769,7 @@
         <v>0.25295075090609098</v>
       </c>
     </row>
-    <row r="192" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>193</v>
       </c>
@@ -17783,7 +17780,7 @@
         <v>0.256452611497334</v>
       </c>
     </row>
-    <row r="193" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>194</v>
       </c>
@@ -17794,7 +17791,7 @@
         <v>0.25868777299010298</v>
       </c>
     </row>
-    <row r="194" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>195</v>
       </c>
@@ -17805,7 +17802,7 @@
         <v>0.2539674766801</v>
       </c>
     </row>
-    <row r="195" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>196</v>
       </c>
@@ -17816,7 +17813,7 @@
         <v>0.17294771128421699</v>
       </c>
     </row>
-    <row r="196" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>197</v>
       </c>
@@ -17827,7 +17824,7 @@
         <v>0.175665485735155</v>
       </c>
     </row>
-    <row r="197" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>198</v>
       </c>
@@ -17838,7 +17835,7 @@
         <v>0.17382778027635701</v>
       </c>
     </row>
-    <row r="198" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>199</v>
       </c>
@@ -17849,7 +17846,7 @@
         <v>0.17455983570099701</v>
       </c>
     </row>
-    <row r="199" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>200</v>
       </c>
@@ -17860,7 +17857,7 @@
         <v>0.17664296551393399</v>
       </c>
     </row>
-    <row r="200" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>201</v>
       </c>
@@ -17871,7 +17868,7 @@
         <v>0.17708531560420199</v>
       </c>
     </row>
-    <row r="201" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>202</v>
       </c>
@@ -17882,7 +17879,7 @@
         <v>0.17557573140333699</v>
       </c>
     </row>
-    <row r="202" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>203</v>
       </c>
@@ -17893,7 +17890,7 @@
         <v>0.173457649972002</v>
       </c>
     </row>
-    <row r="203" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>204</v>
       </c>
@@ -17904,7 +17901,7 @@
         <v>0.17535865105134299</v>
       </c>
     </row>
-    <row r="204" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>205</v>
       </c>
@@ -17915,7 +17912,7 @@
         <v>0.175039518424147</v>
       </c>
     </row>
-    <row r="205" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>206</v>
       </c>
@@ -17926,7 +17923,7 @@
         <v>0.17459939950666101</v>
       </c>
     </row>
-    <row r="206" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>207</v>
       </c>
@@ -17937,7 +17934,7 @@
         <v>0.17177387798819599</v>
       </c>
     </row>
-    <row r="207" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>208</v>
       </c>
@@ -17948,7 +17945,7 @@
         <v>0.172049396498035</v>
       </c>
     </row>
-    <row r="208" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>209</v>
       </c>
@@ -17959,7 +17956,7 @@
         <v>0.17416028353340501</v>
       </c>
     </row>
-    <row r="209" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>210</v>
       </c>
@@ -17970,7 +17967,7 @@
         <v>0.17432866559164001</v>
       </c>
     </row>
-    <row r="210" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>211</v>
       </c>
@@ -17981,7 +17978,7 @@
         <v>0.17371638201273101</v>
       </c>
     </row>
-    <row r="211" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>212</v>
       </c>
@@ -17992,7 +17989,7 @@
         <v>0.17123203171632401</v>
       </c>
     </row>
-    <row r="212" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>213</v>
       </c>
@@ -18003,7 +18000,7 @@
         <v>0.17318569822136001</v>
       </c>
     </row>
-    <row r="213" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>214</v>
       </c>
@@ -18014,7 +18011,7 @@
         <v>0.17669669700448201</v>
       </c>
     </row>
-    <row r="214" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>215</v>
       </c>
@@ -18025,7 +18022,7 @@
         <v>0.17723933870696301</v>
       </c>
     </row>
-    <row r="215" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>216</v>
       </c>
@@ -18036,7 +18033,7 @@
         <v>0.17063092731327101</v>
       </c>
     </row>
-    <row r="216" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>217</v>
       </c>
@@ -18047,7 +18044,7 @@
         <v>0.17490193092626999</v>
       </c>
     </row>
-    <row r="217" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>218</v>
       </c>
@@ -18058,7 +18055,7 @@
         <v>0.17702310390171999</v>
       </c>
     </row>
-    <row r="218" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>219</v>
       </c>
@@ -18069,7 +18066,7 @@
         <v>0.171948853936535</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>220</v>
       </c>
@@ -18080,7 +18077,7 @@
         <v>0.17411860264206899</v>
       </c>
     </row>
-    <row r="220" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>221</v>
       </c>
@@ -18091,7 +18088,7 @@
         <v>0.175935205113702</v>
       </c>
     </row>
-    <row r="221" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>222</v>
       </c>
@@ -18102,7 +18099,7 @@
         <v>0.17427622300988699</v>
       </c>
     </row>
-    <row r="222" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>223</v>
       </c>
@@ -18113,7 +18110,7 @@
         <v>0.17224969239811899</v>
       </c>
     </row>
-    <row r="223" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>224</v>
       </c>
@@ -18124,7 +18121,7 @@
         <v>0.17435257559575301</v>
       </c>
     </row>
-    <row r="224" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>225</v>
       </c>
@@ -18135,7 +18132,7 @@
         <v>0.171222354567128</v>
       </c>
     </row>
-    <row r="225" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>226</v>
       </c>
@@ -18146,7 +18143,7 @@
         <v>0.17230494746765301</v>
       </c>
     </row>
-    <row r="226" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>227</v>
       </c>
@@ -18157,7 +18154,7 @@
         <v>0.17976030708667101</v>
       </c>
     </row>
-    <row r="227" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>228</v>
       </c>
@@ -18168,7 +18165,7 @@
         <v>0.174433801903358</v>
       </c>
     </row>
-    <row r="228" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>229</v>
       </c>
@@ -18179,7 +18176,7 @@
         <v>0.17714435708530099</v>
       </c>
     </row>
-    <row r="229" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>230</v>
       </c>
@@ -18190,7 +18187,7 @@
         <v>0.17086804073973499</v>
       </c>
     </row>
-    <row r="230" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>231</v>
       </c>
@@ -18201,7 +18198,7 @@
         <v>0.171697248433512</v>
       </c>
     </row>
-    <row r="231" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>232</v>
       </c>
@@ -18212,7 +18209,7 @@
         <v>0.17443666559002999</v>
       </c>
     </row>
-    <row r="232" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>233</v>
       </c>
@@ -18223,7 +18220,7 @@
         <v>0.17690051952166999</v>
       </c>
     </row>
-    <row r="233" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>234</v>
       </c>
@@ -18233,6 +18230,254 @@
       <c r="C233" s="1">
         <v>0.17654554655181801</v>
       </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B234" s="1"/>
+      <c r="C234" s="1"/>
+    </row>
+    <row r="235" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B235" s="1"/>
+      <c r="C235" s="1"/>
+    </row>
+    <row r="236" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B236" s="1"/>
+      <c r="C236" s="1"/>
+    </row>
+    <row r="237" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B237" s="1"/>
+      <c r="C237" s="1"/>
+    </row>
+    <row r="238" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B238" s="1"/>
+      <c r="C238" s="1"/>
+    </row>
+    <row r="239" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B239" s="1"/>
+      <c r="C239" s="1"/>
+    </row>
+    <row r="240" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B240" s="1"/>
+      <c r="C240" s="1"/>
+    </row>
+    <row r="241" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B241" s="1"/>
+      <c r="C241" s="1"/>
+    </row>
+    <row r="242" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B242" s="1"/>
+      <c r="C242" s="1"/>
+    </row>
+    <row r="243" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B243" s="1"/>
+      <c r="C243" s="1"/>
+    </row>
+    <row r="244" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B244" s="1"/>
+      <c r="C244" s="1"/>
+    </row>
+    <row r="245" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B245" s="1"/>
+      <c r="C245" s="1"/>
+    </row>
+    <row r="246" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B246" s="1"/>
+      <c r="C246" s="1"/>
+    </row>
+    <row r="247" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B247" s="1"/>
+      <c r="C247" s="1"/>
+    </row>
+    <row r="248" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B248" s="1"/>
+      <c r="C248" s="1"/>
+    </row>
+    <row r="249" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B249" s="1"/>
+      <c r="C249" s="1"/>
+    </row>
+    <row r="250" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B250" s="1"/>
+      <c r="C250" s="1"/>
+    </row>
+    <row r="251" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B251" s="1"/>
+      <c r="C251" s="1"/>
+    </row>
+    <row r="252" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B252" s="1"/>
+      <c r="C252" s="1"/>
+    </row>
+    <row r="253" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B253" s="1"/>
+      <c r="C253" s="1"/>
+    </row>
+    <row r="254" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B254" s="1"/>
+      <c r="C254" s="1"/>
+    </row>
+    <row r="255" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B255" s="1"/>
+      <c r="C255" s="1"/>
+    </row>
+    <row r="256" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B256" s="1"/>
+      <c r="C256" s="1"/>
+    </row>
+    <row r="257" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B257" s="1"/>
+      <c r="C257" s="1"/>
+    </row>
+    <row r="258" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B258" s="1"/>
+      <c r="C258" s="1"/>
+    </row>
+    <row r="259" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B259" s="1"/>
+      <c r="C259" s="1"/>
+    </row>
+    <row r="260" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B260" s="1"/>
+      <c r="C260" s="1"/>
+    </row>
+    <row r="261" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B261" s="1"/>
+      <c r="C261" s="1"/>
+    </row>
+    <row r="262" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B262" s="1"/>
+      <c r="C262" s="1"/>
+    </row>
+    <row r="263" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B263" s="1"/>
+      <c r="C263" s="1"/>
+    </row>
+    <row r="264" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B264" s="1"/>
+      <c r="C264" s="1"/>
+    </row>
+    <row r="265" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B265" s="1"/>
+      <c r="C265" s="1"/>
+    </row>
+    <row r="266" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B266" s="1"/>
+      <c r="C266" s="1"/>
+    </row>
+    <row r="267" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B267" s="1"/>
+      <c r="C267" s="1"/>
+    </row>
+    <row r="268" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B268" s="1"/>
+      <c r="C268" s="1"/>
+    </row>
+    <row r="269" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B269" s="1"/>
+      <c r="C269" s="1"/>
+    </row>
+    <row r="270" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B270" s="1"/>
+      <c r="C270" s="1"/>
+    </row>
+    <row r="271" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B271" s="1"/>
+      <c r="C271" s="1"/>
+    </row>
+    <row r="272" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B272" s="1"/>
+      <c r="C272" s="1"/>
+    </row>
+    <row r="273" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B273" s="1"/>
+      <c r="C273" s="1"/>
+    </row>
+    <row r="274" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B274" s="1"/>
+      <c r="C274" s="1"/>
+    </row>
+    <row r="275" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B275" s="1"/>
+      <c r="C275" s="1"/>
+    </row>
+    <row r="276" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B276" s="1"/>
+      <c r="C276" s="1"/>
+    </row>
+    <row r="277" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B277" s="1"/>
+      <c r="C277" s="1"/>
+    </row>
+    <row r="278" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B278" s="1"/>
+      <c r="C278" s="1"/>
+    </row>
+    <row r="279" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B279" s="1"/>
+      <c r="C279" s="1"/>
+    </row>
+    <row r="280" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B280" s="1"/>
+      <c r="C280" s="1"/>
+    </row>
+    <row r="281" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B281" s="1"/>
+      <c r="C281" s="1"/>
+    </row>
+    <row r="282" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B282" s="1"/>
+      <c r="C282" s="1"/>
+    </row>
+    <row r="283" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B283" s="1"/>
+      <c r="C283" s="1"/>
+    </row>
+    <row r="284" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B284" s="1"/>
+      <c r="C284" s="1"/>
+    </row>
+    <row r="285" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B285" s="1"/>
+      <c r="C285" s="1"/>
+    </row>
+    <row r="286" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B286" s="1"/>
+      <c r="C286" s="1"/>
+    </row>
+    <row r="287" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B287" s="1"/>
+      <c r="C287" s="1"/>
+    </row>
+    <row r="288" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B288" s="1"/>
+      <c r="C288" s="1"/>
+    </row>
+    <row r="289" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B289" s="1"/>
+      <c r="C289" s="1"/>
+    </row>
+    <row r="290" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B290" s="1"/>
+      <c r="C290" s="1"/>
+    </row>
+    <row r="291" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B291" s="1"/>
+      <c r="C291" s="1"/>
+    </row>
+    <row r="292" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B292" s="1"/>
+      <c r="C292" s="1"/>
+    </row>
+    <row r="293" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B293" s="1"/>
+      <c r="C293" s="1"/>
+    </row>
+    <row r="294" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B294" s="1"/>
+      <c r="C294" s="1"/>
+    </row>
+    <row r="295" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B295" s="1"/>
+      <c r="C295" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18243,13 +18488,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D318508-EB39-4B19-9441-3235666F09D0}">
   <dimension ref="A1:K39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>246</v>
       </c>
@@ -18294,7 +18539,7 @@
         <v>1.2279085192200808E-3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>247</v>
       </c>
@@ -18339,7 +18584,7 @@
         <v>0.70533132928470998</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>245</v>
       </c>
@@ -18374,7 +18619,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
@@ -18409,7 +18654,7 @@
         <v>0.17086804073973499</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2</v>
       </c>
@@ -18444,7 +18689,7 @@
         <v>0.171697248433512</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>3</v>
       </c>
@@ -18479,7 +18724,7 @@
         <v>0.17443666559002999</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>4</v>
       </c>
@@ -18514,7 +18759,7 @@
         <v>0.17690051952166999</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>5</v>
       </c>
@@ -18549,7 +18794,7 @@
         <v>0.17654554655181801</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>6</v>
       </c>
@@ -18578,7 +18823,7 @@
         <v>0.17411860264206899</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>7</v>
       </c>
@@ -18607,7 +18852,7 @@
         <v>0.175935205113702</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>8</v>
       </c>
@@ -18636,7 +18881,7 @@
         <v>0.17427622300988699</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>9</v>
       </c>
@@ -18665,7 +18910,7 @@
         <v>0.17224969239811899</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>10</v>
       </c>
@@ -18694,7 +18939,7 @@
         <v>0.17435257559575301</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>11</v>
       </c>
@@ -18723,7 +18968,7 @@
         <v>0.171222354567128</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>12</v>
       </c>
@@ -18752,7 +18997,7 @@
         <v>0.17230494746765301</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>13</v>
       </c>
@@ -18781,7 +19026,7 @@
         <v>0.17976030708667101</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>14</v>
       </c>
@@ -18810,7 +19055,7 @@
         <v>0.174433801903358</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>15</v>
       </c>
@@ -18839,7 +19084,7 @@
         <v>0.17714435708530099</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>16</v>
       </c>
@@ -18865,7 +19110,7 @@
         <v>0.17371638201273101</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>17</v>
       </c>
@@ -18888,7 +19133,7 @@
         <v>0.17123203171632401</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>18</v>
       </c>
@@ -18911,7 +19156,7 @@
         <v>0.17318569822136001</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>19</v>
       </c>
@@ -18934,7 +19179,7 @@
         <v>0.17669669700448201</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>20</v>
       </c>
@@ -18954,7 +19199,7 @@
         <v>0.25295075090609098</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>21</v>
       </c>
@@ -18971,7 +19216,7 @@
         <v>0.256452611497334</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>22</v>
       </c>
@@ -18988,7 +19233,7 @@
         <v>0.25868777299010298</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>23</v>
       </c>
@@ -19005,7 +19250,7 @@
         <v>0.2539674766801</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>24</v>
       </c>
@@ -19019,7 +19264,7 @@
         <v>0.25848980394328103</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>25</v>
       </c>
@@ -19033,7 +19278,7 @@
         <v>0.25493042534243598</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>26</v>
       </c>
@@ -19047,7 +19292,7 @@
         <v>0.25702073078272197</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>27</v>
       </c>
@@ -19061,7 +19306,7 @@
         <v>0.25281370286486299</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>28</v>
       </c>
@@ -19075,7 +19320,7 @@
         <v>0.25787828139437702</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>29</v>
       </c>
@@ -19089,7 +19334,7 @@
         <v>0.255030114263046</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>30</v>
       </c>
@@ -19103,7 +19348,7 @@
         <v>0.25326708245889501</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>31</v>
       </c>
@@ -19117,7 +19362,7 @@
         <v>0.25901851572451601</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>32</v>
       </c>
@@ -19128,7 +19373,7 @@
         <v>0.22249606599096799</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>33</v>
       </c>
@@ -19136,7 +19381,7 @@
         <v>0.22770140189949001</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>34</v>
       </c>
@@ -19144,7 +19389,7 @@
         <v>0.22467693879523801</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>35</v>
       </c>
@@ -19152,7 +19397,7 @@
         <v>0.22590951148508701</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>36</v>
       </c>
@@ -19170,12 +19415,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A5AE877-64C3-4028-8147-765389663D58}">
   <dimension ref="A1:K39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>246</v>
       </c>
@@ -19220,7 +19465,7 @@
         <v>5.1155359965755959E-2</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>247</v>
       </c>
@@ -19265,7 +19510,7 @@
         <v>0.47681214118341592</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>245</v>
       </c>
@@ -19300,7 +19545,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
@@ -19335,7 +19580,7 @@
         <v>10.6539096425895</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2</v>
       </c>
@@ -19370,7 +19615,7 @@
         <v>10.8579810008815</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>3</v>
       </c>
@@ -19405,7 +19650,7 @@
         <v>10.831312443746899</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>4</v>
       </c>
@@ -19440,7 +19685,7 @@
         <v>10.709515833036701</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>5</v>
       </c>
@@ -19475,7 +19720,7 @@
         <v>10.5903781690852</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>6</v>
       </c>
@@ -19504,7 +19749,7 @@
         <v>10.753363759575</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>7</v>
       </c>
@@ -19533,7 +19778,7 @@
         <v>10.653749196664901</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>8</v>
       </c>
@@ -19562,7 +19807,7 @@
         <v>10.8630753057798</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>9</v>
       </c>
@@ -19591,7 +19836,7 @@
         <v>10.7208205400928</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>10</v>
       </c>
@@ -19620,7 +19865,7 @@
         <v>10.6700806810118</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>11</v>
       </c>
@@ -19649,7 +19894,7 @@
         <v>10.6606574449491</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>12</v>
       </c>
@@ -19678,7 +19923,7 @@
         <v>10.8131728102025</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>13</v>
       </c>
@@ -19707,7 +19952,7 @@
         <v>10.8081420366551</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>14</v>
       </c>
@@ -19736,7 +19981,7 @@
         <v>10.586819027671799</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>15</v>
       </c>
@@ -19765,7 +20010,7 @@
         <v>10.7337029456849</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>16</v>
       </c>
@@ -19791,7 +20036,7 @@
         <v>10.7080767594852</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>17</v>
       </c>
@@ -19814,7 +20059,7 @@
         <v>10.6292015876151</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>18</v>
       </c>
@@ -19837,7 +20082,7 @@
         <v>10.6922490647235</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>19</v>
       </c>
@@ -19860,7 +20105,7 @@
         <v>10.661460418557301</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>20</v>
       </c>
@@ -19880,7 +20125,7 @@
         <v>15.924948044130501</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>21</v>
       </c>
@@ -19897,7 +20142,7 @@
         <v>15.963192712237699</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>22</v>
       </c>
@@ -19914,7 +20159,7 @@
         <v>15.8676552218831</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>23</v>
       </c>
@@ -19931,7 +20176,7 @@
         <v>15.928435989248699</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>24</v>
       </c>
@@ -19945,7 +20190,7 @@
         <v>15.4712021433598</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>25</v>
       </c>
@@ -19959,7 +20204,7 @@
         <v>15.4267437621642</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>26</v>
       </c>
@@ -19973,7 +20218,7 @@
         <v>15.363023447442201</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>27</v>
       </c>
@@ -19987,7 +20232,7 @@
         <v>15.4784018893041</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>28</v>
       </c>
@@ -20001,7 +20246,7 @@
         <v>15.598700910453401</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>29</v>
       </c>
@@ -20015,7 +20260,7 @@
         <v>15.699463941581101</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>30</v>
       </c>
@@ -20029,7 +20274,7 @@
         <v>15.751226314712399</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>31</v>
       </c>
@@ -20043,7 +20288,7 @@
         <v>15.601321813860199</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>32</v>
       </c>
@@ -20054,7 +20299,7 @@
         <v>13.9597270287277</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>33</v>
       </c>
@@ -20062,7 +20307,7 @@
         <v>13.946102058433601</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>34</v>
       </c>
@@ -20070,7 +20315,7 @@
         <v>13.9823014618208</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>35</v>
       </c>
@@ -20078,7 +20323,7 @@
         <v>13.749906400784599</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
Almost Done, Need to fit total Data
</commit_message>
<xml_diff>
--- a/BeatnotePostHotCell/AllFitsF1=3_playing with.xlsx
+++ b/BeatnotePostHotCell/AllFitsF1=3_playing with.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\BeatnotePostHotCell\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CB86C3-BC88-4521-946B-C38277BB1D8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{276BDF60-ADE8-4023-A979-AE706728F51E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Together" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="346">
   <si>
     <t>Date</t>
   </si>
@@ -1002,6 +1002,81 @@
   </si>
   <si>
     <t>Jun29,2026+6-02-58PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+10-01-11AM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+11-04-27AM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+12-29-37PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+12-50-34PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+12-58-35PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+1-42-43PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+2-04-26PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+2-13-49PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+2-44-43PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+2-53-14PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+3-01-33PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+3-10-00PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+3-18-31PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+3-37-15PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+3-50-02PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+3-58-54PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+4-08-15PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+4-16-19PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+4-25-35PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+4-33-28PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+4-42-00PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+4-49-59PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+4-59-09PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+5-07-22PM</t>
+  </si>
+  <si>
+    <t>Jul02,2026+9-53-21AM</t>
   </si>
 </sst>
 </file>
@@ -7131,6 +7206,245 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-5A79-43C7-A012-327EE2E82A5E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>2-Jun</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'All Together'!$B$299:$B$329</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>14.824645793302301</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14.4528707103913</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>14.6109532885724</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>14.525535608882601</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>14.703570164436799</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>14.6469605754983</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>14.4430203101595</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>14.549598435905899</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>14.7043335718615</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>14.770828981153199</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>14.7903674498711</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>14.6129136258226</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>14.5285253520751</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14.4495865267067</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>14.524765784844201</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>14.764112552014099</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>14.7106184874969</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>14.749177714501</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>14.6684970880551</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>14.5764121579489</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>14.633716179029699</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>14.618198212113001</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>14.482642723981799</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>14.491750683935599</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>14.610387851091801</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>16.418772327555299</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>16.352237501405199</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>16.311710862235199</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>16.368589028451201</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>16.289962255694199</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>16.347944436289598</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'All Together'!$C$299:$C$329</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>0.24180291421483799</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.23775144209915899</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.24065215342237201</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.238634580986853</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.24123516367901099</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.23838761262462899</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.23787175668006799</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.235957408677299</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.23761103430247099</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.24049928819975</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.23875237313230799</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.23577509684512599</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.23798590162913699</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.23776270729380899</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.23525871098023601</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.23822698567085801</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.236137249858582</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.236589149526167</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.234995035195148</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.238435257488993</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.23631298859917599</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.238968925765909</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.237506075673066</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.237718713583811</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.23747635372092801</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.26184487099436499</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.26409583467590397</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.26424448419416702</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.26363414452799</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.26464837628465498</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.27030866825799199</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-98E0-4FAF-A3DC-7EEEAA62D55C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -18121,15 +18435,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>853656</xdr:colOff>
-      <xdr:row>256</xdr:row>
-      <xdr:rowOff>503207</xdr:rowOff>
+      <xdr:colOff>485235</xdr:colOff>
+      <xdr:row>291</xdr:row>
+      <xdr:rowOff>143772</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>530165</xdr:colOff>
-      <xdr:row>268</xdr:row>
-      <xdr:rowOff>122804</xdr:rowOff>
+      <xdr:colOff>161744</xdr:colOff>
+      <xdr:row>303</xdr:row>
+      <xdr:rowOff>149760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -18576,7 +18890,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P298"/>
+  <dimension ref="A1:P329"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="16.140625" customWidth="1"/>
@@ -21957,6 +22271,347 @@
     <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B298" s="1"/>
       <c r="C298" s="1"/>
+    </row>
+    <row r="299" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A299" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="B299" s="1">
+        <v>14.824645793302301</v>
+      </c>
+      <c r="C299" s="1">
+        <v>0.24180291421483799</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A300" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="B300" s="1">
+        <v>14.4528707103913</v>
+      </c>
+      <c r="C300" s="1">
+        <v>0.23775144209915899</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A301" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="B301" s="1">
+        <v>14.6109532885724</v>
+      </c>
+      <c r="C301" s="1">
+        <v>0.24065215342237201</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A302" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B302" s="1">
+        <v>14.525535608882601</v>
+      </c>
+      <c r="C302" s="1">
+        <v>0.238634580986853</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A303" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="B303" s="1">
+        <v>14.703570164436799</v>
+      </c>
+      <c r="C303" s="1">
+        <v>0.24123516367901099</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A304" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="B304" s="1">
+        <v>14.6469605754983</v>
+      </c>
+      <c r="C304" s="1">
+        <v>0.23838761262462899</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A305" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B305" s="1">
+        <v>14.4430203101595</v>
+      </c>
+      <c r="C305" s="1">
+        <v>0.23787175668006799</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A306" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B306" s="1">
+        <v>14.549598435905899</v>
+      </c>
+      <c r="C306" s="1">
+        <v>0.235957408677299</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A307" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="B307" s="1">
+        <v>14.7043335718615</v>
+      </c>
+      <c r="C307" s="1">
+        <v>0.23761103430247099</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A308" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="B308" s="1">
+        <v>14.770828981153199</v>
+      </c>
+      <c r="C308" s="1">
+        <v>0.24049928819975</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A309" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B309" s="1">
+        <v>14.7903674498711</v>
+      </c>
+      <c r="C309" s="1">
+        <v>0.23875237313230799</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A310" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="B310" s="1">
+        <v>14.6129136258226</v>
+      </c>
+      <c r="C310" s="1">
+        <v>0.23577509684512599</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A311" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="B311" s="1">
+        <v>14.5285253520751</v>
+      </c>
+      <c r="C311" s="1">
+        <v>0.23798590162913699</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A312" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B312" s="1">
+        <v>14.4495865267067</v>
+      </c>
+      <c r="C312" s="1">
+        <v>0.23776270729380899</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A313" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B313" s="1">
+        <v>14.524765784844201</v>
+      </c>
+      <c r="C313" s="1">
+        <v>0.23525871098023601</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A314" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="B314" s="1">
+        <v>14.764112552014099</v>
+      </c>
+      <c r="C314" s="1">
+        <v>0.23822698567085801</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A315" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B315" s="1">
+        <v>14.7106184874969</v>
+      </c>
+      <c r="C315" s="1">
+        <v>0.236137249858582</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A316" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B316" s="1">
+        <v>14.749177714501</v>
+      </c>
+      <c r="C316" s="1">
+        <v>0.236589149526167</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A317" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B317" s="1">
+        <v>14.6684970880551</v>
+      </c>
+      <c r="C317" s="1">
+        <v>0.234995035195148</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A318" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="B318" s="1">
+        <v>14.5764121579489</v>
+      </c>
+      <c r="C318" s="1">
+        <v>0.238435257488993</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A319" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="B319" s="1">
+        <v>14.633716179029699</v>
+      </c>
+      <c r="C319" s="1">
+        <v>0.23631298859917599</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A320" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="B320" s="1">
+        <v>14.618198212113001</v>
+      </c>
+      <c r="C320" s="1">
+        <v>0.238968925765909</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A321" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="B321" s="1">
+        <v>14.482642723981799</v>
+      </c>
+      <c r="C321" s="1">
+        <v>0.237506075673066</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A322" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="B322" s="1">
+        <v>14.491750683935599</v>
+      </c>
+      <c r="C322" s="1">
+        <v>0.237718713583811</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A323" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B323" s="1">
+        <v>14.610387851091801</v>
+      </c>
+      <c r="C323" s="1">
+        <v>0.23747635372092801</v>
+      </c>
+    </row>
+    <row r="324" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A324" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="B324" s="1">
+        <v>16.418772327555299</v>
+      </c>
+      <c r="C324" s="1">
+        <v>0.26184487099436499</v>
+      </c>
+    </row>
+    <row r="325" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A325" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B325" s="1">
+        <v>16.352237501405199</v>
+      </c>
+      <c r="C325" s="1">
+        <v>0.26409583467590397</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A326" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B326" s="1">
+        <v>16.311710862235199</v>
+      </c>
+      <c r="C326" s="1">
+        <v>0.26424448419416702</v>
+      </c>
+    </row>
+    <row r="327" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A327" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B327" s="1">
+        <v>16.368589028451201</v>
+      </c>
+      <c r="C327" s="1">
+        <v>0.26363414452799</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A328" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="B328" s="1">
+        <v>16.289962255694199</v>
+      </c>
+      <c r="C328" s="1">
+        <v>0.26464837628465498</v>
+      </c>
+    </row>
+    <row r="329" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A329" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="B329" s="1">
+        <v>16.347944436289598</v>
+      </c>
+      <c r="C329" s="1">
+        <v>0.27030866825799199</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>